<commit_message>
bom und fehler behebung von nicht aktiven bauteilen- 3h
</commit_message>
<xml_diff>
--- a/Hardware/PCB_Project/DIP_V01_Testing/PCB_Project/Project Outputs for PCB_Project/PCB_Project.xlsx
+++ b/Hardware/PCB_Project/DIP_V01_Testing/PCB_Project/Project Outputs for PCB_Project/PCB_Project.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micha\Documents\Messung_von_Quanteneffecten_in_MOSFETs\Diplom_Arbeit\Hardware\PCB_Project\DIP_V01_Testing\PCB_Project\Project Outputs for PCB_Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Michael Watzek\Documents\Diplom_Arbeit\Hardware\PCB_Project\DIP_V01_Testing\PCB_Project\Project Outputs for PCB_Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{71F430B0-A7F3-4A97-8CAD-3D986A560F33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8524CC6B-7128-4E68-8E06-CA7A97FDFE2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="3444" windowWidth="23040" windowHeight="12120" xr2:uid="{DCA40F51-8512-4217-A924-FE98D5DE5A30}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{082D1CAA-8991-464C-8581-E7ED76C5CE06}"/>
   </bookViews>
   <sheets>
     <sheet name="PCB_Project" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="121">
   <si>
     <t>Comment</t>
   </si>
@@ -77,13 +77,13 @@
     <t>100nF</t>
   </si>
   <si>
-    <t>C2, C3, C4, C5, C11, C13, C14, C16, C17, C18, C20, C22, C24, C29, C31, C34, C37, C39, C41, C43, C48, C50, C54, C55</t>
+    <t>C2, C3, C4, C5, C11, C13, C14, C16, C17, C18, C34, C37, C39, C41, C43, C48, C50, C54, C55</t>
   </si>
   <si>
     <t>10uF</t>
   </si>
   <si>
-    <t>C6, C8, C10, C12, C15, C27, C32, C33, C35, C45, C46, C47, C49, C51, C52</t>
+    <t>C6, C8, C10, C12, C15, C27, C35, C45, C46, C47, C49, C51, C52</t>
   </si>
   <si>
     <t>4.7uF</t>
@@ -95,7 +95,13 @@
     <t>1uF</t>
   </si>
   <si>
-    <t>C19, C21, C23, C25, C26, C30, C38, C40, C42, C44, C53</t>
+    <t>C25, C26, C38, C40, C42, C44, C53</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>C29</t>
   </si>
   <si>
     <t>GREEN</t>
@@ -167,9 +173,6 @@
     <t>STM32F103</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>N4</t>
   </si>
   <si>
@@ -206,36 +209,12 @@
     <t>Header, 2-Pin</t>
   </si>
   <si>
-    <t>P5, P8, P10, P11, P12</t>
+    <t>P5, P10, P11, P12</t>
   </si>
   <si>
     <t>HDR1X2</t>
   </si>
   <si>
-    <t>472192001</t>
-  </si>
-  <si>
-    <t>1.10mm Pitch microSD Card Connector, Hinge Type, Lead-Free</t>
-  </si>
-  <si>
-    <t>P6</t>
-  </si>
-  <si>
-    <t>CONN_47219-2001_MOL</t>
-  </si>
-  <si>
-    <t>Header 6X2</t>
-  </si>
-  <si>
-    <t>Header, 6-Pin, Dual row</t>
-  </si>
-  <si>
-    <t>P7</t>
-  </si>
-  <si>
-    <t>HDR2X6</t>
-  </si>
-  <si>
     <t>CNS020-10MP</t>
   </si>
   <si>
@@ -257,7 +236,7 @@
     <t>Resistor SMD</t>
   </si>
   <si>
-    <t>R2, R9, R14, R15, R25, R26, R28, R29, R31, R32, R34, R36, R37, R38, R45, R46</t>
+    <t>R2, R9, R14, R15, R34, R36, R37, R38, R45, R46</t>
   </si>
   <si>
     <t>ResistorSMD</t>
@@ -296,19 +275,19 @@
     <t>4.7k</t>
   </si>
   <si>
-    <t>R11, R12, R13, R17, R18, R19, R23, R24, R27, R30, R39</t>
+    <t>R11, R12, R13, R39</t>
   </si>
   <si>
     <t>3.9k</t>
   </si>
   <si>
-    <t>R16, R20</t>
+    <t>R16, R17</t>
   </si>
   <si>
     <t>2.7k</t>
   </si>
   <si>
-    <t>R21</t>
+    <t>R18</t>
   </si>
   <si>
     <t>49.9k</t>
@@ -371,15 +350,6 @@
     <t>RU_16_ADI</t>
   </si>
   <si>
-    <t>APS6404L-3SQR-SN</t>
-  </si>
-  <si>
-    <t>U4, U5, U6</t>
-  </si>
-  <si>
-    <t>APS6404L-3SQR-SN_APY</t>
-  </si>
-  <si>
     <t>OPA197IDBVR</t>
   </si>
   <si>
@@ -410,7 +380,7 @@
     <t>Adjustable- and fixed-output, 1-A, 16-V, positive-voltage low-dropout (LDO) linear regulator 8-HVSSOP -40 to 125</t>
   </si>
   <si>
-    <t>U11, U12</t>
+    <t>U12</t>
   </si>
   <si>
     <t>VSSOP8_DGN_TEX</t>
@@ -830,11 +800,13 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD4FE00A-820F-4123-8419-D37E974F9CDE}">
-  <dimension ref="A1:F39"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F6C343A-6375-4B56-977D-967D0FE7D3FC}">
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="6" width="19.44140625" customWidth="1"/>
+    <col min="1" max="1" width="19.44140625" customWidth="1"/>
+    <col min="2" max="2" width="54.5546875" customWidth="1"/>
+    <col min="3" max="6" width="19.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -894,7 +866,7 @@
         <v>7</v>
       </c>
       <c r="F3" s="1">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -914,7 +886,7 @@
         <v>7</v>
       </c>
       <c r="F4" s="1">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -954,7 +926,7 @@
         <v>7</v>
       </c>
       <c r="F6" s="1">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -962,39 +934,39 @@
         <v>18</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="D7" s="2" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="F7" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="F8" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -1002,76 +974,76 @@
         <v>25</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F9" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>30</v>
-      </c>
       <c r="E10" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F10" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>34</v>
-      </c>
       <c r="E11" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="F11" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="F12" s="1">
         <v>1</v>
@@ -1079,19 +1051,19 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>43</v>
-      </c>
       <c r="E13" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F13" s="1">
         <v>1</v>
@@ -1099,99 +1071,99 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>47</v>
-      </c>
       <c r="E14" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F14" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>51</v>
-      </c>
       <c r="E15" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F15" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>55</v>
-      </c>
       <c r="E16" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F16" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="E17" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F17" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>60</v>
       </c>
       <c r="F18" s="1">
         <v>1</v>
@@ -1199,59 +1171,59 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="D19" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>68</v>
-      </c>
       <c r="F19" s="1">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F20" s="1">
-        <v>16</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F21" s="1">
         <v>1</v>
@@ -1259,139 +1231,139 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F22" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F23" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F24" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F25" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F26" s="1">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F27" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F28" s="1">
         <v>1</v>
@@ -1399,19 +1371,19 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>9</v>
+        <v>87</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="F29" s="1">
         <v>1</v>
@@ -1419,59 +1391,59 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="E30" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>91</v>
-      </c>
       <c r="F30" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="D31" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="E31" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>99</v>
-      </c>
       <c r="F31" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="D32" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C32" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>103</v>
-      </c>
       <c r="E32" s="2" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="F32" s="1">
         <v>1</v>
@@ -1479,141 +1451,101 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D33" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>108</v>
-      </c>
       <c r="E33" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="F33" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="E34" s="2" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F34" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="D35" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="C35" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>115</v>
-      </c>
       <c r="E35" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F35" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>119</v>
-      </c>
       <c r="E36" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F36" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>123</v>
-      </c>
       <c r="E37" s="2" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="F37" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="F38" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="F39" s="1">
         <v>1</v>
       </c>
     </row>

</xml_diff>